<commit_message>
found a UB matrix for Alex's crystal
</commit_message>
<xml_diff>
--- a/wombat_alex_crystal_example/Alex_crystal_structure_factors.xlsx
+++ b/wombat_alex_crystal_example/Alex_crystal_structure_factors.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="J:\wombat_instrument_work\eulerian_cradle\Wombat_DMCpy\wombat_alex_crystal_example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C1D9FBD-0420-4BE7-8A36-F37E51247CB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89830C1C-C2F5-4C99-AD60-7843463FCAD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25365" yWindow="1785" windowWidth="21600" windowHeight="12510" xr2:uid="{9D007949-E7B7-4C00-B4CB-B92E7A23D255}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{9D007949-E7B7-4C00-B4CB-B92E7A23D255}"/>
   </bookViews>
   <sheets>
     <sheet name="alex_crystal_cool_5_30093_high_" sheetId="2" r:id="rId1"/>

</xml_diff>